<commit_message>
improved kanban cards during drag-drop process
</commit_message>
<xml_diff>
--- a/workspace/data/MY_DataBase.xlsx
+++ b/workspace/data/MY_DataBase.xlsx
@@ -7008,7 +7008,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17 00:00:00</t>
+          <t>2026-03-19 14:44:18</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Operations/Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 00:00:00</t>
+          <t>2026-03-19 14:44:21</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17 00:00:00</t>
+          <t>2026-03-19 14:44:22</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 08:58:24</t>
+          <t>2026-03-19 14:42:17</t>
         </is>
       </c>
     </row>
@@ -7521,7 +7521,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Operations/Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 08:58:24</t>
+          <t>2026-03-19 14:42:16</t>
         </is>
       </c>
     </row>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -7593,7 +7593,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 08:58:24</t>
+          <t>2026-03-19 14:42:14</t>
         </is>
       </c>
     </row>
@@ -28708,42 +28708,42 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>P_FMS-HYB_FUEL_MANAGEMENT_SYSTEM_HYBRID_V1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>FMS-HYB</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Fuel Management System Hybrid v1</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Hybrid AC/DC fuel management system.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>2025-12-20 00:00:00</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>2026-03-19 14:06:55</t>
         </is>

</xml_diff>

<commit_message>
merged with kanban drag-drop fix
</commit_message>
<xml_diff>
--- a/workspace/data/MY_DataBase.xlsx
+++ b/workspace/data/MY_DataBase.xlsx
@@ -3582,7 +3582,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 00:00:00</t>
+          <t>2026-03-19 14:45:39</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -3655,12 +3655,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 12:00:33</t>
+          <t>2026-03-19 14:45:39</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Electrical/Automation</t>
+          <t>Fabrication</t>
         </is>
       </c>
       <c r="H47" s="2" t="n">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 18:11:36</t>
+          <t>2026-03-19 14:45:59</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Electrical/Automation</t>
+          <t>Fabrication</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -5565,7 +5565,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 18:11:37</t>
+          <t>2026-03-19 14:45:59</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Operations/Assembly</t>
+          <t>Fabrication</t>
         </is>
       </c>
       <c r="H49" s="2" t="n">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 18:11:37</t>
+          <t>2026-03-19 14:45:59</t>
         </is>
       </c>
     </row>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 14:44:18</t>
+          <t>2026-03-19 14:46:16</t>
         </is>
       </c>
     </row>
@@ -33820,7 +33820,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>2026-03-17 00:00:00</t>
+          <t>2026-03-19 14:45:39</t>
         </is>
       </c>
     </row>
@@ -34473,7 +34473,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -34493,7 +34493,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 18:11:35</t>
+          <t>2026-03-19 14:45:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
completed jobs now showing successfully
</commit_message>
<xml_diff>
--- a/workspace/data/MY_DataBase.xlsx
+++ b/workspace/data/MY_DataBase.xlsx
@@ -21,6 +21,8 @@
     <sheet name="WorkOrders" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="README" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Parts" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="CompletedJobs" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="CompletedJobLines" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -10197,6 +10199,1775 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="24" customWidth="1" style="3" min="1" max="1"/>
+    <col width="22" customWidth="1" style="3" min="2" max="2"/>
+    <col width="28" customWidth="1" style="3" min="3" max="3"/>
+    <col width="32" customWidth="1" style="3" min="4" max="4"/>
+    <col width="18" customWidth="1" style="3" min="5" max="5"/>
+    <col width="18" customWidth="1" style="3" min="6" max="6"/>
+    <col width="20" customWidth="1" style="3" min="7" max="7"/>
+    <col width="24" customWidth="1" style="3" min="8" max="8"/>
+    <col width="18" customWidth="1" style="3" min="9" max="9"/>
+    <col width="18" customWidth="1" style="3" min="10" max="10"/>
+    <col width="18" customWidth="1" style="3" min="11" max="11"/>
+    <col width="18" customWidth="1" style="3" min="12" max="12"/>
+    <col width="18" customWidth="1" style="3" min="13" max="13"/>
+    <col width="18" customWidth="1" style="3" min="14" max="14"/>
+    <col width="18" customWidth="1" style="3" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>SnapshotID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>ProjectCode</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>QuoteRef</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>ProductCode</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>ProductName</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>ClientName</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>CompletedOn</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>LabourHours</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>PartsTotal</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>GrandTotal</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>OQ-008</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PROD-016</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Steel Frame Kiosk</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Client 08</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 14:54:18</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Frozen snapshot created on completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>OQ-004</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>PROD-004</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Standpipe 8 inch</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Client 04</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 14:54:19</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Frozen snapshot created on completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>OQ-003</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>PROD-003</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Standpipe 6 inch</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Client 03</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 14:54:20</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Frozen snapshot created on completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OQ-001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PROD-001</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Standpipe 2 inch</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Client 01</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-03-19 14:54:20</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Frozen snapshot created on completion.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="24" customWidth="1" style="3" min="1" max="1"/>
+    <col width="22" customWidth="1" style="3" min="2" max="2"/>
+    <col width="28" customWidth="1" style="3" min="3" max="3"/>
+    <col width="32" customWidth="1" style="3" min="4" max="4"/>
+    <col width="18" customWidth="1" style="3" min="5" max="5"/>
+    <col width="18" customWidth="1" style="3" min="6" max="6"/>
+    <col width="20" customWidth="1" style="3" min="7" max="7"/>
+    <col width="24" customWidth="1" style="3" min="8" max="8"/>
+    <col width="18" customWidth="1" style="3" min="9" max="9"/>
+    <col width="18" customWidth="1" style="3" min="10" max="10"/>
+    <col width="18" customWidth="1" style="3" min="11" max="11"/>
+    <col width="18" customWidth="1" style="3" min="12" max="12"/>
+    <col width="18" customWidth="1" style="3" min="13" max="13"/>
+    <col width="18" customWidth="1" style="3" min="14" max="14"/>
+    <col width="18" customWidth="1" style="3" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>SnapshotLineID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>SnapshotID</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>LineType</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>PartNumber</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>UnitPrice</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>LineTotal</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418-ASM-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ASM-027</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ASM-027</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418-ASM-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ASM-014</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ASM-014</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418-PART-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Control Panel Door</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Control Panel Door</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418-PART-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-008_FUEL_MANAGEMENT_SYSTEM_AC_ORDER_8::20260319145418</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Panel Cooling Fan</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Panel Cooling Fan</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-ASM-001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ASM-007</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ASM-007</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-ASM-002</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ASM-008</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>ASM-008</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-003</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Pipe 8 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Pipe 8 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-004</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Stub 8 inch</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Stub 8 inch</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-005</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-006</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31 00:00:00</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-007</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419-PART-008</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-004_STANDPIPE_8_INCH_ORDER_4::20260319145419</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Flange 8 inch</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Flange 8 inch</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-ASM-001</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ASM-005</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ASM-005</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-ASM-002</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ASM-006</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>ASM-006</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-003</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Pipe 6 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Pipe 6 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-004</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Stub 6 inch</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Stub 6 inch</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-005</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-006</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-007</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-008</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Flange 6 inch</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Flange 6 inch</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420-PART-009</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-003_STANDPIPE_6_INCH_ORDER_3::20260319145420</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>AC Contactor</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>AC Contactor</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-ASM-001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ASM-001</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ASM-001</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-ASM-002</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ASM-002</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ASM-002</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PRODUCT_MODULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-003</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pipe 2 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Pipe 2 inch 6 meters</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-12-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-004</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Stub 2 inch</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Stub 2 inch</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-02-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-005</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Poly Hinge</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-01-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-006</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Bolt M12 Galv</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-01-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-007</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Lug 12mm</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420-PART-008</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SNAP::PRJ_OQ-001_STANDPIPE_2_INCH_ORDER_1::20260319145420</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Flange 2 inch</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Flange 2 inch</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2025-12-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PRODUCT_DIRECT_PART</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -33007,7 +34778,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>PROD-008</t>
+          <t>PROD-016</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -33032,7 +34803,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-03-18 18:11:34</t>
+          <t>2026-03-19 14:50:21</t>
         </is>
       </c>
     </row>

</xml_diff>